<commit_message>
Enhanced PA generation with detailed KPIs and NWU values, improved teaching outputs summarization, and fixed enrollment functionality
</commit_message>
<xml_diff>
--- a/backend/data/performance_agreements/PA_20172672_2025_web.xlsx
+++ b/backend/data/performance_agreements/PA_20172672_2025_web.xlsx
@@ -66,32 +66,59 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Teaching and Learning</t>
+          <t>Teaching and Learning (including supervision)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t/>
+          <t>• Lesson planning, assessment design, learning outcomes | Modules: HISE411 (85 students), HISE312 (25 students), HISE321 (100 students), SSCE321 (97 students), ERTP 671 (1 students), LERP 671 (1 students)
+• eFundi configuration, content upload, resource preparation | Modules: HISE411 (85 students), HISE312 (25 students), HISE321 (100 students), SSCE321 (97 students), ERTP 671 (1 students), LERP 671 (1 students)
+• Study guide updates, reading list compilation, material preparation | Modules: HISE411 (85 students), HISE312 (25 students), HISE321 (100 students), SSCE321 (97 students), ERTP 671 (1 students), LERP 671 (1 students)
+• Assessment calendar, rubrics, marking criteria | Modules: HISE411 (85 students), HISE312 (25 students), HISE321 (100 students), SSCE321 (97 students), ERTP 671 (1 students), LERP 671 (1 students)
+• Orientation week &amp; student onboarding | First lectures | Class lists &amp; student consultation setup | Modules: HISE411 (85 students), HISE312 (25 students)
+• Regular lectures &amp; tutorials | Formative assessments &amp; feedback | Student consultations | Modules: HISE411 (85 students), HISE312 (25 students)
+• Mid-term assessments &amp; tests | Student feedback sessions | Remedial interventions | Modules: HISE411 (85 students), HISE312 (25 students)
+• Final lectures &amp; exam prep | Semester tests &amp; assignments | Exam prep workshops | Modules: HISE411 (85 students), HISE312 (25 students)
+• Exam invigilation | Exam marking &amp; moderation | Grade submission &amp; finalization | Modules: HISE411 (85 students), HISE312 (25 students)
+• Semester 2 planning &amp; prep | Module revisions &amp; updates | Research time allocation | Modules: HISE411 (85 students), HISE312 (25 students), HISE321 (100 students), SSCE321 (97 students), ERTP 671 (1 students), LERP 671 (1 students)
+• Welcome back sessions | Semester 2 lectures begin | Assessment schedules distribution | Modules: HISE321 (100 students), SSCE321 (97 students)
+• Regular lectures &amp; tutorials | Formative assessments | Student consultations | Modules: HISE321 (100 students), SSCE321 (97 students)
+• Mid-term assessments | Student feedback &amp; interventions | Remedial support | Modules: HISE321 (100 students), SSCE321 (97 students)
+• Final lectures &amp; reviews | Semester tests | Exam prep workshops | Modules: HISE321 (100 students), SSCE321 (97 students)
+• Exam invigilation | Final marking &amp; moderation | Grade finalization | Modules: HISE321 (100 students), SSCE321 (97 students)
+• Semester 1 assessment completion for HISE411 (85 students), HISE312 (25 students), HISE321 (100 students), SSCE321 (97 students), ERTP 671 (1 students), LERP 671 (1 students)
+• Year-end assessment completion and moderation for HISE411 (85 students), HISE312 (25 students), HISE321 (100 students), SSCE321 (97 students), ERTP 671 (1 students), LERP 671 (1 students)
+• Module evaluation and improvement for HISE411 (85 students), HISE312 (25 students), HISE321 (100 students), SSCE321 (97 students), ERTP 671 (1 students), LERP 671 (1 students)
+• Teaching practice supervision and assessment for April window
+• Teaching practice supervision and assessment for July window
+• Preparation for ROR: Presentation: 1 hour per presentation times  number of presentations divided by number of presenters
+• ROR programme delivery: Presentation: 1 hour per presentation times  number of presentations divided by number of presenters</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Curriculum delivery
-Assessment &amp; feedback
-LMS (eFundi) management
-Moderation
-Student support</t>
+          <t>STLES results (Student Teaching and Learning Evaluation Surveys)
+Peer reviews of teaching (e.g., observation reports)
+eFundi LMS activity reports
+Teaching portfolios, including reflective narratives
+Pass and throughput rates for modules taught
+Curriculum development (e.g., new modules, curriculum renewal)
+Contact hours and module credits
+Teaching awards (e.g., Institutional Teaching Excellence Award - ITEA)
+Assessment and moderation compliance (aligned with NWU's policy)
+Supervision of undergraduate and honours students
+Use of innovative pedagogy, such as blended or AI-assisted learning</t>
         </is>
       </c>
       <c r="D3">
-        <v>0.0</v>
+        <v>52.41</v>
       </c>
       <c r="E3">
-        <v>0.0</v>
+        <v>811.742</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Excellence; Innovation; Integrity; Social Responsiveness</t>
+          <t>Excellence; Ethics; Unity in Diversity; Human Dignity; Commitment; Self-Respect; Respect for Others; Accountability; Transparency; Innovation; Social Responsiveness; Collaboration; Lifelong Learning; Environmental Stewardship; Service Orientation</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -103,32 +130,49 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Research and Innovation / Creative Outputs</t>
+          <t>Personal Research, Innovation and/or Creative Outputs</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t/>
+          <t>• Citesaga project
+• WorkReady Project
+• AI and GBL project
+• GBL conference
+• Article on AI GBL
+• Article on Citesaga project
+• Article on WorkReady project
+• Prosper book chapter
+• Attendance of research colloquiums, writing schools, workshops (eg. Ethics, Integrity, Turnitin): Maximum of 60 hours
+• NRF funding application or rating improvement
+• Research publication submission or conference acceptance
+• Accredited research publication for subsidy purposes
+• Students: Rensberg, MED | Choba, MED | Temo, MED | Olivier | van Deventer</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>IRIMS updates
-Manuscript pipeline
-Grant applications
-Supervision
-Conference dissemination</t>
+          <t>DHET-accredited journal articles (with ISSN/DOI)
+Conference papers (national or international)
+Books or book chapters (accredited)
+NRF rating status (e.g., Y1, C2)
+Research funding/grants (applications and awards)
+Research supervision (Master's and PhD graduations)
+Ethics approval letters (REC/HREC)
+Innovation outputs (e.g., patents, software, creative works)
+Research awards or commendations
+Editorial board membership or invited keynote talks</t>
         </is>
       </c>
       <c r="D4">
-        <v>0.0</v>
+        <v>33.9</v>
       </c>
       <c r="E4">
-        <v>0.0</v>
+        <v>525.0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Excellence; Innovation; Integrity; Social Responsiveness</t>
+          <t>Excellence; Ethics; Unity in Diversity; Human Dignity; Commitment; Self-Respect; Respect for Others; Accountability; Transparency; Innovation; Social Responsiveness; Collaboration; Lifelong Learning; Environmental Stewardship; Service Orientation</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -140,7 +184,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Social Responsiveness / Community and Industry Engagement</t>
+          <t>Social Responsiveness (Community Engagement / Industry)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -150,10 +194,15 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Community engagement
-Partnerships
-Outreach reporting
-Media/impact</t>
+          <t>Registered community engagement projects
+Service-learning initiatives in curriculum
+Public lectures or science engagement activities
+Signed MoUs with NGOs, schools, or local government
+Community-based research with impact reports
+Media participation (e.g., radio, TV, newspapers)
+Recognition or awards for societal impact
+Advisory board or committee service
+Volunteer work using academic expertise</t>
         </is>
       </c>
       <c r="D5">
@@ -164,7 +213,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Excellence; Innovation; Integrity; Social Responsiveness</t>
+          <t>Excellence; Ethics; Unity in Diversity; Human Dignity; Commitment; Self-Respect; Respect for Others; Accountability; Transparency; Innovation; Social Responsiveness; Collaboration; Lifelong Learning; Environmental Stewardship; Service Orientation</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -176,31 +225,46 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Academic Leadership and Management</t>
+          <t>Academic Leadership and Administration</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t/>
+          <t>• Research Focus Area/Entity meetings: Maximum of 10 hours
+• Mentorship meetings: 8 hours
+• School Management Committee: 24 hours
+• Subject Group meetings: 22 hours
+• School meetings and functions: 10 hours
+• Faculty Forums: Maximum of 6 hours
+• Professional development (in accordance with PDP): Maximum of 10 hours
+• Staff performance reviews and development planning
+• Year-end performance review, annual achievements summary, and next year planning
+• Module leadership for HISE 411, HISE322: Monthly reports, assessment planning, cross-campus coordination
+• Programme accreditation documentation and quality reviews</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Committee participation
-Chairing/secretariat
-Workplan execution
-Governance compliance</t>
+          <t>Head of Department, Program Leader, or Entity Director roles
+Faculty or institutional committee membership
+Mentorship of junior academics or tutors
+Accreditation or re-accreditation reports led
+Strategic planning or policy input
+Development and management of academic programs
+Performance management of reporting staff
+Leadership in transformation or equity initiatives
+Meeting minutes or official project documentation</t>
         </is>
       </c>
       <c r="D6">
-        <v>0.0</v>
+        <v>13.56</v>
       </c>
       <c r="E6">
-        <v>0.0</v>
+        <v>210.0</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Excellence; Innovation; Integrity; Social Responsiveness</t>
+          <t>Excellence; Ethics; Unity in Diversity; Human Dignity; Commitment; Self-Respect; Respect for Others; Accountability; Transparency; Innovation; Social Responsiveness; Collaboration; Lifelong Learning; Environmental Stewardship; Service Orientation</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -212,7 +276,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Occupational Health and Safety</t>
+          <t>Occupational Health &amp; Safety</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -222,22 +286,25 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Annual OHS compliance
-Incident reporting
-Safety training
-Risk assessment
-Drills</t>
+          <t>Completed OHS training/induction (mandatory NWU modules)
+Risk assessment documents for labs, fieldwork, and events
+Zero-incident reports for labs or teaching spaces
+Incident reporting records (if applicable)
+Participation in OHS committees or audits
+Evidence of student OHS induction
+Compliance with COVID-19 or pandemic protocols
+Use of NWU OHS tools (e.g., digital safety platforms)</t>
         </is>
       </c>
       <c r="D7">
-        <v>2.0</v>
+        <v>0.13</v>
       </c>
       <c r="E7">
         <v>2.0</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Excellence; Innovation; Integrity; Social Responsiveness</t>
+          <t>Excellence; Ethics; Unity in Diversity; Human Dignity; Commitment; Self-Respect; Respect for Others; Accountability; Transparency; Innovation; Social Responsiveness; Collaboration; Lifelong Learning; Environmental Stewardship; Service Orientation</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">

</xml_diff>